<commit_message>
Defect Register v0.6 and Open Items v0.8: RC evidence filled in (DEF-007 to DEF-012 fixed in #136, DEF-019 closed, OI-13 closed with evidence, CON-019 final)
</commit_message>
<xml_diff>
--- a/docs/Requirements/Open Items/Open_Items_v0.8.xlsx
+++ b/docs/Requirements/Open Items/Open_Items_v0.8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SEN381\Repo\Ticketing-System\docs\Requirements\Open Items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77383712-11EB-4D9C-A9B4-09A89DEBBE50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815D6F83-FA82-40CC-9E76-B9DD3683BFD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="164">
   <si>
     <t>Open Items &amp; Assumptions</t>
   </si>
@@ -406,9 +406,6 @@
     <t>Raised 13/10/2026 by R. van der Merwe, found when asked to deploy; recorded by E. Lindsay. Related: R. van der Merwe (DEC-003 owner), DEC-002</t>
   </si>
   <si>
-    <t>Gaps, derived requirements and unvalidated figures carried by this baseline. Recorded rather than resolved by invention — Master Brief s.23 values honest limitations above unsupported claims of completeness | Version 0.8 (17/10/2026, M4 final pass, R. van der Merwe). Adds columns I (Final status, M4: Closed with evidence, or Remains open for future work) and J (the engineering reason and the evidence). Every open item is given a final status. OI-05, OI-06, OI-09, OI-11 and OI-19 were closed earlier and are left exactly as they were. Adds two rows for items carried from M2 that are not open items but need a final status here: C-05 (PED Appendix B) and CON-019. E. Lindsay's two new items (the missing category list; the Information Officer in AC-NFR-4.5) are inserted after OI-21, with the IDs and text he allocates. Columns B to H of every existing row are unchanged. Version 0.7 (13/10/2026). Closes OI-19 (DEC-003 v0.3, PR #92, records the test environment's name, Atlas project and redacted cluster hostname separately, and the integration-test guard cites it), raised by E. Lindsay. Adds OI-21 (DEC-003 places staging and production on a VPS that never existed; found at deployment and resolved for staging only by a disposable Azure VM, with DEC-003 to be superseded), raised by R. van der Merwe. OI-01 to OI-18 and OI-20 unchanged. Version 0.6 (12/10/2026; OI-20 added 13/10/2026). Adds OI-17 (the read endpoint refuses the whole read of a security-category request to non-Security-Officer staff, which is wider than FR-1.5's three restricted fields), OI-18 (whether a blank or whitespace-only reason counts as a recorded reason under FR-6.6), OI-19 (DEC-003 names the test environment's Atlas project civicconnect-test, but the test cluster's host and the integration-test guard use civicconnecttest) and OI-20 (no CI gate inspects content inside non-Office binaries such as images and PDFs; found when an embedded provenance manifest in the three PED architecture figures passed every required check, removed on PR #94), all raised by E. Lindsay; OI-01 to OI-16 unchanged. Version 0.5 (30/09/2026). Adds OI-16 (FR-1.5 against FR-3.5/FR-3.6: whether a requester may see their own description on a security-category request), raised by E. Lindsay; OI-01 to OI-15 unchanged. Version 0.4 (30/09/2026). Adds OI-14 (reportingCounts reconciliation, owner R. van der Merwe for M3) and OI-15 (transition model confirmation, including whether a reopened-then-resolved request satisfies FR-6.5), both raised in PR #62 (E. Lindsay) and its review (R. van der Merwe). OI-01 to OI-13 are unchanged from v0.3. Version 0.3 (29/09/2026). Consolidates the M2 updates drafted by E. Lindsay (OI-05 closed; OI-06 escalated; OI-07, OI-10 updated; OI-12 raised), first committed inside the file named Open_Items_v0.2 (archived in Outdated/ and carrying those v0.3 labels), with the DEC-017 and storage updates by R. van der Merwe (OI-06 closed, OI-10 reduced, OI-13 raised). No separately committed v0.2 content exists in the repository.</t>
-  </si>
-  <si>
     <t>Final status (M4)</t>
   </si>
   <si>
@@ -442,9 +439,6 @@
     <t>The one-month period was never confirmed with STK-009, and no institutional retention standard was cited. It stays a team position, and the NFR-4.2 basis says so. Evidence: Decision Log v0.10, DEC-005.</t>
   </si>
   <si>
-    <t>Remains open for future work [Sunday RC check: CR-003's final status from PED v4.0]</t>
-  </si>
-  <si>
     <t>CR-003, the PROC-001 exception to FR-6.7, was still Proposed at v3.0-M3-baseline (PED v3.0 M3.10), so FR-6.7 and NFR-4.2 still conflict as written after day 30. PROC-001 is run by hand only (scripts/retention/proc-001-anonymise.js). If PED v4.0 records CR-003 as approved, this item closes with that as evidence.</t>
   </si>
   <si>
@@ -511,10 +505,13 @@
     <t>M3 (PED v3.0 M3.10); owner C. Burger for the tests</t>
   </si>
   <si>
-    <t>Remains open for future work [Sunday RC check: whether E2E-2 or any adversarial case was run against staging at v4.0-M4-rc]</t>
-  </si>
-  <si>
-    <t>Partly evidenced, not met. A route-table test fails CI if a non-public route lacks the guard (NFR-3.3). E2E-2 calls the API directly with a wrong role and is refused with nothing written, but at M3 it ran locally only. Nothing has probed the deployed staging server. Login has no throttling (RSK-021, CodeQL #1), and the field-level restriction is not built (OI-16). Encryption at rest is not evidenced (NFR-3.7). Evidence: tests/authorisationGuard.test.js; docs/evidence/M3-e2e/; DEC-003 v0.5.</t>
+    <t>Gaps, derived requirements and unvalidated figures carried by this baseline. Recorded rather than resolved by invention — Master Brief s.23 values honest limitations above unsupported claims of completeness | Version 0.8 (17/10/2026, M4 final pass, R. van der Merwe). Adds columns I (Final status, M4: Closed with evidence, or Remains open for future work) and J (the engineering reason and the evidence). Every open item is given a final status. OI-05, OI-06, OI-09, OI-11 and OI-19 were closed earlier and are left exactly as they were. Adds two rows for items carried from M2 that are not open items but need a final status here: C-05 (PED Appendix B) and CON-019. E. Lindsay's two new items (the missing category list; the Information Officer in AC-NFR-4.5) are inserted after OI-21, with the IDs and text he allocates. On 18/10/2026 OI-13 was closed with evidence (CR-003 approved, PR #137) and CON-019's final status confirmed from the v4.0-M4-rc evidence. Columns B to H of every existing row are unchanged. Version 0.7 (13/10/2026). Closes OI-19 (DEC-003 v0.3, PR #92, records the test environment's name, Atlas project and redacted cluster hostname separately, and the integration-test guard cites it), raised by E. Lindsay. Adds OI-21 (DEC-003 places staging and production on a VPS that never existed; found at deployment and resolved for staging only by a disposable Azure VM, with DEC-003 to be superseded), raised by R. van der Merwe. OI-01 to OI-18 and OI-20 unchanged. Version 0.6 (12/10/2026; OI-20 added 13/10/2026). Adds OI-17 (the read endpoint refuses the whole read of a security-category request to non-Security-Officer staff, which is wider than FR-1.5's three restricted fields), OI-18 (whether a blank or whitespace-only reason counts as a recorded reason under FR-6.6), OI-19 (DEC-003 names the test environment's Atlas project civicconnect-test, but the test cluster's host and the integration-test guard use civicconnecttest) and OI-20 (no CI gate inspects content inside non-Office binaries such as images and PDFs; found when an embedded provenance manifest in the three PED architecture figures passed every required check, removed on PR #94), all raised by E. Lindsay; OI-01 to OI-16 unchanged. Version 0.5 (30/09/2026). Adds OI-16 (FR-1.5 against FR-3.5/FR-3.6: whether a requester may see their own description on a security-category request), raised by E. Lindsay; OI-01 to OI-15 unchanged. Version 0.4 (30/09/2026). Adds OI-14 (reportingCounts reconciliation, owner R. van der Merwe for M3) and OI-15 (transition model confirmation, including whether a reopened-then-resolved request satisfies FR-6.5), both raised in PR #62 (E. Lindsay) and its review (R. van der Merwe). OI-01 to OI-13 are unchanged from v0.3. Version 0.3 (29/09/2026). Consolidates the M2 updates drafted by E. Lindsay (OI-05 closed; OI-06 escalated; OI-07, OI-10 updated; OI-12 raised), first committed inside the file named Open_Items_v0.2 (archived in Outdated/ and carrying those v0.3 labels), with the DEC-017 and storage updates by R. van der Merwe (OI-06 closed, OI-10 reduced, OI-13 raised). No separately committed v0.2 content exists in the repository.</t>
+  </si>
+  <si>
+    <t>Closed with evidence</t>
+  </si>
+  <si>
+    <t>Partly evidenced, not met. A route-table test fails CI if a non-public route lacks the guard (NFR-3.3). E2E-2 calls the API directly with a wrong role and is refused with nothing written, but at M3 it ran locally only. Nothing has probed the deployed staging server: no adversarial case ran on staging at v4.0-M4-rc (18/10/2026), where the checks were TLS, the performance log, stored passwords and session and query plans. Login has no throttling (RSK-021, CodeQL #1), and the field-level restriction is not built (OI-16). Encryption at rest is not evidenced (NFR-3.7). Evidence: tests/authorisationGuard.test.js; docs/evidence/M3-e2e/; DEC-003 v0.5.</t>
   </si>
 </sst>
 </file>
@@ -997,7 +994,7 @@
     </row>
     <row r="2" spans="2:10" ht="82.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
-        <v>128</v>
+        <v>161</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -1029,13 +1026,13 @@
         <v>7</v>
       </c>
       <c r="I4" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="J4" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="2:10" ht="71.25" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
         <v>8</v>
       </c>
@@ -1058,13 +1055,13 @@
         <v>14</v>
       </c>
       <c r="I5" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="2:10" ht="57" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
         <v>15</v>
       </c>
@@ -1087,13 +1084,13 @@
         <v>14</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="57" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
         <v>20</v>
       </c>
@@ -1116,13 +1113,13 @@
         <v>14</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
         <v>24</v>
       </c>
@@ -1145,10 +1142,10 @@
         <v>30</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="9" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
@@ -1197,7 +1194,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="2:10" ht="399" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
         <v>44</v>
       </c>
@@ -1220,13 +1217,13 @@
         <v>14</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="12" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
       <c r="B12" s="10" t="s">
         <v>49</v>
       </c>
@@ -1249,10 +1246,10 @@
         <v>14</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="2:10" ht="57" x14ac:dyDescent="0.25">
@@ -1278,7 +1275,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" ht="171" x14ac:dyDescent="0.25">
       <c r="B14" s="10" t="s">
         <v>61</v>
       </c>
@@ -1301,10 +1298,10 @@
         <v>30</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="2:10" ht="57" x14ac:dyDescent="0.25">
@@ -1330,7 +1327,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="2:10" ht="399" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" ht="114" x14ac:dyDescent="0.25">
       <c r="B16" s="11" t="s">
         <v>72</v>
       </c>
@@ -1353,13 +1350,13 @@
         <v>14</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" ht="105" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>77</v>
       </c>
@@ -1382,13 +1379,13 @@
         <v>14</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>140</v>
+        <v>162</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" ht="105" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>83</v>
       </c>
@@ -1411,13 +1408,13 @@
         <v>89</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="19" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" ht="225" x14ac:dyDescent="0.25">
       <c r="B19" s="4" t="s">
         <v>90</v>
       </c>
@@ -1440,13 +1437,13 @@
         <v>14</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B20" s="4" t="s">
         <v>96</v>
       </c>
@@ -1469,13 +1466,13 @@
         <v>14</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="21" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" ht="150" x14ac:dyDescent="0.25">
       <c r="B21" s="4" t="s">
         <v>102</v>
       </c>
@@ -1498,13 +1495,13 @@
         <v>14</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="22" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" ht="120" x14ac:dyDescent="0.25">
       <c r="B22" s="4" t="s">
         <v>107</v>
       </c>
@@ -1527,10 +1524,10 @@
         <v>14</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="23" spans="2:10" ht="345" x14ac:dyDescent="0.25">
@@ -1556,7 +1553,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="24" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:10" ht="210" x14ac:dyDescent="0.25">
       <c r="B24" s="4" t="s">
         <v>115</v>
       </c>
@@ -1579,13 +1576,13 @@
         <v>14</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="25" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10" ht="330" x14ac:dyDescent="0.25">
       <c r="B25" s="4" t="s">
         <v>123</v>
       </c>
@@ -1608,68 +1605,68 @@
         <v>14</v>
       </c>
       <c r="I25" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" ht="120" x14ac:dyDescent="0.25">
+      <c r="B26" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="J25" s="8" t="s">
+      <c r="C26" s="8" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="26" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="B26" s="4" t="s">
+      <c r="D26" s="8" t="s">
         <v>150</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="E26" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="F26" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="G26" s="8" t="s">
         <v>153</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>155</v>
       </c>
       <c r="H26" s="8" t="s">
         <v>14</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J26" s="8" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" ht="165" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="C27" s="8" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="27" spans="2:10" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="B27" s="4" t="s">
+      <c r="D27" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="E27" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="F27" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="G27" s="8" t="s">
         <v>160</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>161</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>162</v>
       </c>
       <c r="H27" s="8" t="s">
         <v>14</v>
       </c>
       <c r="I27" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="J27" s="8" t="s">
         <v>163</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Defect Register v0.6: DEF-022 to DEF-031 (fixed in #136) and DEF-032 (counter contention, S1, P2, Open) from E. Lindsay's rows; DEF-019 P29 and O29; Open Items v0.8: OI-13 J17 in E. Lindsay's wording, version note
</commit_message>
<xml_diff>
--- a/docs/Requirements/Open Items/Open_Items_v0.8.xlsx
+++ b/docs/Requirements/Open Items/Open_Items_v0.8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SEN381\Repo\Ticketing-System\docs\Requirements\Open Items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{815D6F83-FA82-40CC-9E76-B9DD3683BFD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C10202-C40E-49F6-80F7-8E7D29AC0019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -439,9 +439,6 @@
     <t>The one-month period was never confirmed with STK-009, and no institutional retention standard was cited. It stays a team position, and the NFR-4.2 basis says so. Evidence: Decision Log v0.10, DEC-005.</t>
   </si>
   <si>
-    <t>CR-003, the PROC-001 exception to FR-6.7, was still Proposed at v3.0-M3-baseline (PED v3.0 M3.10), so FR-6.7 and NFR-4.2 still conflict as written after day 30. PROC-001 is run by hand only (scripts/retention/proc-001-anonymise.js). If PED v4.0 records CR-003 as approved, this item closes with that as evidence.</t>
-  </si>
-  <si>
     <t>No reconciliation job was built, and the M3 target was missed (owner R. van der Merwe). The reportingCounts subscriber is not registered (TD-001), so the projection is not maintained at all yet. Nothing drifts, but reporting (feature group 8) is not built either. scripts/backup/consistency-check.js exists for the restore path but is not scheduled. Evidence: TD-001 (Technical Debt Register); PED v3.0 M3.10.</t>
   </si>
   <si>
@@ -505,13 +502,16 @@
     <t>M3 (PED v3.0 M3.10); owner C. Burger for the tests</t>
   </si>
   <si>
-    <t>Gaps, derived requirements and unvalidated figures carried by this baseline. Recorded rather than resolved by invention — Master Brief s.23 values honest limitations above unsupported claims of completeness | Version 0.8 (17/10/2026, M4 final pass, R. van der Merwe). Adds columns I (Final status, M4: Closed with evidence, or Remains open for future work) and J (the engineering reason and the evidence). Every open item is given a final status. OI-05, OI-06, OI-09, OI-11 and OI-19 were closed earlier and are left exactly as they were. Adds two rows for items carried from M2 that are not open items but need a final status here: C-05 (PED Appendix B) and CON-019. E. Lindsay's two new items (the missing category list; the Information Officer in AC-NFR-4.5) are inserted after OI-21, with the IDs and text he allocates. On 18/10/2026 OI-13 was closed with evidence (CR-003 approved, PR #137) and CON-019's final status confirmed from the v4.0-M4-rc evidence. Columns B to H of every existing row are unchanged. Version 0.7 (13/10/2026). Closes OI-19 (DEC-003 v0.3, PR #92, records the test environment's name, Atlas project and redacted cluster hostname separately, and the integration-test guard cites it), raised by E. Lindsay. Adds OI-21 (DEC-003 places staging and production on a VPS that never existed; found at deployment and resolved for staging only by a disposable Azure VM, with DEC-003 to be superseded), raised by R. van der Merwe. OI-01 to OI-18 and OI-20 unchanged. Version 0.6 (12/10/2026; OI-20 added 13/10/2026). Adds OI-17 (the read endpoint refuses the whole read of a security-category request to non-Security-Officer staff, which is wider than FR-1.5's three restricted fields), OI-18 (whether a blank or whitespace-only reason counts as a recorded reason under FR-6.6), OI-19 (DEC-003 names the test environment's Atlas project civicconnect-test, but the test cluster's host and the integration-test guard use civicconnecttest) and OI-20 (no CI gate inspects content inside non-Office binaries such as images and PDFs; found when an embedded provenance manifest in the three PED architecture figures passed every required check, removed on PR #94), all raised by E. Lindsay; OI-01 to OI-16 unchanged. Version 0.5 (30/09/2026). Adds OI-16 (FR-1.5 against FR-3.5/FR-3.6: whether a requester may see their own description on a security-category request), raised by E. Lindsay; OI-01 to OI-15 unchanged. Version 0.4 (30/09/2026). Adds OI-14 (reportingCounts reconciliation, owner R. van der Merwe for M3) and OI-15 (transition model confirmation, including whether a reopened-then-resolved request satisfies FR-6.5), both raised in PR #62 (E. Lindsay) and its review (R. van der Merwe). OI-01 to OI-13 are unchanged from v0.3. Version 0.3 (29/09/2026). Consolidates the M2 updates drafted by E. Lindsay (OI-05 closed; OI-06 escalated; OI-07, OI-10 updated; OI-12 raised), first committed inside the file named Open_Items_v0.2 (archived in Outdated/ and carrying those v0.3 labels), with the DEC-017 and storage updates by R. van der Merwe (OI-06 closed, OI-10 reduced, OI-13 raised). No separately committed v0.2 content exists in the repository.</t>
-  </si>
-  <si>
     <t>Closed with evidence</t>
   </si>
   <si>
     <t>Partly evidenced, not met. A route-table test fails CI if a non-public route lacks the guard (NFR-3.3). E2E-2 calls the API directly with a wrong role and is refused with nothing written, but at M3 it ran locally only. Nothing has probed the deployed staging server: no adversarial case ran on staging at v4.0-M4-rc (18/10/2026), where the checks were TLS, the performance log, stored passwords and session and query plans. Login has no throttling (RSK-021, CodeQL #1), and the field-level restriction is not built (OI-16). Encryption at rest is not evidenced (NFR-3.7). Evidence: tests/authorisationGuard.test.js; docs/evidence/M3-e2e/; DEC-003 v0.5.</t>
+  </si>
+  <si>
+    <t>Closed by CR-003, approved 17/10/2026 by the team (E. Lindsay, Team Lead) at M4 closure; not validated with a client stakeholder. FR-6.7's measurement basis (Functional Requirements v0.3) now states the one sanctioned exception: removing personal fields at the end of the retention period under PROC-001 is not an alteration of lifecycle content (status values, change types, roles, timestamps and sequence are preserved), and it is executed only by a temporary, audited database credential outside the system's interfaces. FR-6.7's text and AC-FR-6.7 are unchanged, so FR-6.7 and NFR-4.2 no longer conflict as written. PROC-001 is still run by hand only (scripts/retention/proc-001-anonymise.js; SCP-020 deferred). Evidence: docs/change/CR-003_FR-6.7_Retention_Exception_v0.2.md; PED v4.0.</t>
+  </si>
+  <si>
+    <t>Gaps, derived requirements and unvalidated figures carried by this baseline. Recorded rather than resolved by invention — Master Brief s.23 values honest limitations above unsupported claims of completeness | Version 0.8 (17/10/2026, M4 final pass, R. van der Merwe). Adds columns I (Final status, M4: Closed with evidence, or Remains open for future work) and J (the engineering reason and the evidence). Every open item is given a final status. OI-05, OI-06, OI-09, OI-11 and OI-19 were closed earlier and are left exactly as they were. Adds two rows for items carried from M2 that are not open items but need a final status here: C-05 (PED Appendix B) and CON-019. E. Lindsay's two proposed items (the missing category list; the Information Officer in AC-NFR-4.5) were not raised in this version. On 18/10/2026 OI-13 was closed with evidence (CR-003 approved, PR #137; J17 in E. Lindsay's wording) and CON-019's final status confirmed from the v4.0-M4-rc evidence. Columns B to H of every existing row are unchanged. Version 0.7 (13/10/2026). Closes OI-19 (DEC-003 v0.3, PR #92, records the test environment's name, Atlas project and redacted cluster hostname separately, and the integration-test guard cites it), raised by E. Lindsay. Adds OI-21 (DEC-003 places staging and production on a VPS that never existed; found at deployment and resolved for staging only by a disposable Azure VM, with DEC-003 to be superseded), raised by R. van der Merwe. OI-01 to OI-18 and OI-20 unchanged. Version 0.6 (12/10/2026; OI-20 added 13/10/2026). Adds OI-17 (the read endpoint refuses the whole read of a security-category request to non-Security-Officer staff, which is wider than FR-1.5's three restricted fields), OI-18 (whether a blank or whitespace-only reason counts as a recorded reason under FR-6.6), OI-19 (DEC-003 names the test environment's Atlas project civicconnect-test, but the test cluster's host and the integration-test guard use civicconnecttest) and OI-20 (no CI gate inspects content inside non-Office binaries such as images and PDFs; found when an embedded provenance manifest in the three PED architecture figures passed every required check, removed on PR #94), all raised by E. Lindsay; OI-01 to OI-16 unchanged. Version 0.5 (30/09/2026). Adds OI-16 (FR-1.5 against FR-3.5/FR-3.6: whether a requester may see their own description on a security-category request), raised by E. Lindsay; OI-01 to OI-15 unchanged. Version 0.4 (30/09/2026). Adds OI-14 (reportingCounts reconciliation, owner R. van der Merwe for M3) and OI-15 (transition model confirmation, including whether a reopened-then-resolved request satisfies FR-6.5), both raised in PR #62 (E. Lindsay) and its review (R. van der Merwe). OI-01 to OI-13 are unchanged from v0.3. Version 0.3 (29/09/2026). Consolidates the M2 updates drafted by E. Lindsay (OI-05 closed; OI-06 escalated; OI-07, OI-10 updated; OI-12 raised), first committed inside the file named Open_Items_v0.2 (archived in Outdated/ and carrying those v0.3 labels), with the DEC-017 and storage updates by R. van der Merwe (OI-06 closed, OI-10 reduced, OI-13 raised). No separately committed v0.2 content exists in the repository.</t>
   </si>
 </sst>
 </file>
@@ -994,7 +994,7 @@
     </row>
     <row r="2" spans="2:10" ht="82.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="15" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
@@ -1356,7 +1356,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="2:10" ht="105" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" ht="195" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
         <v>77</v>
       </c>
@@ -1379,10 +1379,10 @@
         <v>14</v>
       </c>
       <c r="I17" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="J17" s="8" t="s">
         <v>162</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="18" spans="2:10" ht="105" x14ac:dyDescent="0.25">
@@ -1411,7 +1411,7 @@
         <v>130</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="225" x14ac:dyDescent="0.25">
@@ -1440,7 +1440,7 @@
         <v>130</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="20" spans="2:10" ht="90" x14ac:dyDescent="0.25">
@@ -1469,7 +1469,7 @@
         <v>130</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="2:10" ht="150" x14ac:dyDescent="0.25">
@@ -1498,7 +1498,7 @@
         <v>130</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" spans="2:10" ht="120" x14ac:dyDescent="0.25">
@@ -1527,7 +1527,7 @@
         <v>130</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="23" spans="2:10" ht="345" x14ac:dyDescent="0.25">
@@ -1579,7 +1579,7 @@
         <v>130</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="25" spans="2:10" ht="330" x14ac:dyDescent="0.25">
@@ -1605,30 +1605,30 @@
         <v>14</v>
       </c>
       <c r="I25" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="J25" s="8" t="s">
         <v>146</v>
-      </c>
-      <c r="J25" s="8" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="26" spans="2:10" ht="120" x14ac:dyDescent="0.25">
       <c r="B26" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="D26" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="D26" s="8" t="s">
+      <c r="E26" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="F26" s="8" t="s">
         <v>151</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="G26" s="8" t="s">
         <v>152</v>
-      </c>
-      <c r="G26" s="8" t="s">
-        <v>153</v>
       </c>
       <c r="H26" s="8" t="s">
         <v>14</v>
@@ -1637,27 +1637,27 @@
         <v>130</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="27" spans="2:10" ht="165" x14ac:dyDescent="0.25">
       <c r="B27" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C27" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="D27" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="D27" s="8" t="s">
+      <c r="E27" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="E27" s="9" t="s">
+      <c r="F27" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="G27" s="8" t="s">
         <v>159</v>
-      </c>
-      <c r="G27" s="8" t="s">
-        <v>160</v>
       </c>
       <c r="H27" s="8" t="s">
         <v>14</v>
@@ -1666,7 +1666,7 @@
         <v>130</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Defect Register v0.6 review fixes: DEF-003 secret-scan history stated accurately (Q13), P29 Fixed, C31 as a DATE formula; Open Items v0.8: OI-02, OI-03, OI-04, OI-07, OI-14 and OI-18 reasons brought up to the M4 build and RC results
</commit_message>
<xml_diff>
--- a/docs/Requirements/Open Items/Open_Items_v0.8.xlsx
+++ b/docs/Requirements/Open Items/Open_Items_v0.8.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SEN381\Repo\Ticketing-System\docs\Requirements\Open Items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C10202-C40E-49F6-80F7-8E7D29AC0019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794F71B9-ED5A-4A46-BB1E-A89613B2D7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -418,18 +418,6 @@
     <t>No SCP ID was added for 'view full request details', and FR-4.2 is still traced provisionally to SCP-005 (Scope Baseline v0.3). A request-detail read exists (GET /api/v1/requests/{id}, OI-17), but the scope-baseline gap this item records was never corrected by Member A. Evidence: Scope Baseline v0.3; RTM v0.11, FR-4.2 row.</t>
   </si>
   <si>
-    <t>Reporting (feature group 8) was not built, and no target resolution time per category was recorded, so overdue requests cannot be computed. The gap did not block anything that was built. Evidence: RTM v0.11 (FR-8.4 status); Scope Baseline v0.3.</t>
-  </si>
-  <si>
-    <t>Category administration (FR-9.1) was not built, and categories exist only as data: a change needs a database write, not a release, but there is no interface for it. Related: E. Lindsay's new item on the missing category list. Evidence: RTM v0.11 (FR-9.1 status); src/models/Category.js.</t>
-  </si>
-  <si>
-    <t>The response-time targets (3 s, 2 s, 5 s) and the 99 % availability figure were never confirmed with STK-005 or STK-010. Only NFR-2.4 was tested, against its own criterion: PASS on staging, 100 users for 600 s with 0 failures (15/10/2026, PED M3.8). NFR-2.1, NFR-2.3 and NFR-2.5 were not measured. Evidence: docs/evidence/M3-perf/NFR-2.4_load_run_2026-10-15.txt.</t>
-  </si>
-  <si>
-    <t>The BC Desktop browser set was never confirmed. E2E runs on Chromium only (DEC-019), so NFR-1.1 browser coverage is not claimed. Evidence: e2e/playwright.config.js; Decision Log v0.10, DEC-013 and DEC-019.</t>
-  </si>
-  <si>
     <t>The SCP-017 to SCP-019 renumbering was never confirmed as deliberate, and no controlled change records it: CR-001 to CR-004 cover other items. Documents citing those IDs may still cite a different capability than when they were written. Evidence: docs/change/ (no CR for the renumbering).</t>
   </si>
   <si>
@@ -439,9 +427,6 @@
     <t>The one-month period was never confirmed with STK-009, and no institutional retention standard was cited. It stays a team position, and the NFR-4.2 basis says so. Evidence: Decision Log v0.10, DEC-005.</t>
   </si>
   <si>
-    <t>No reconciliation job was built, and the M3 target was missed (owner R. van der Merwe). The reportingCounts subscriber is not registered (TD-001), so the projection is not maintained at all yet. Nothing drifts, but reporting (feature group 8) is not built either. scripts/backup/consistency-check.js exists for the restore path but is not scheduled. Evidence: TD-001 (Technical Debt Register); PED v3.0 M3.10.</t>
-  </si>
-  <si>
     <t>The transition model is still a team proposal, not confirmed with the stakeholders. The reopen rule (FR-6.5) and judgements (1) to (4) were not decided. DEF-019's fix corrected the Administrator test's title to cite this item rather than FR-6.7 (PR #123), so the record no longer presents the proposal as baselined. Evidence: src/domain/requestStatus.js header; PR #123.</t>
   </si>
   <si>
@@ -451,9 +436,6 @@
     <t>Not decided. The whole read of a security-category request is still refused to staff who are not Security Officers: more restrictive than FR-1.5, which is the safe direction. Option (b) needs the serialiser, which waits on OI-16. Evidence: src/domain/accessRules.js (mayViewRequest); Decision Log v0.10, DEC-012.</t>
   </si>
   <si>
-    <t>Not decided. As at dev on 17/10/2026, a whitespace-only reason is still accepted: hasReason is Boolean(reason) (src/services/statusTransitionService.js line 80). Consequence: a rejection can carry a reason that tells the requester nothing (FR-3.4). Evidence: that line; AC-FR-6.6.</t>
-  </si>
-  <si>
     <t>No CI gate inspects metadata or text inside images or PDFs. The secret scan covers text and the extracted text of Office documents only, and ci.yml says so. The three figures found on 13/10/2026 were cleaned (PR #94). Evidence: .github/workflows/ci.yml (secret-scan job comments); PR #94.</t>
   </si>
   <si>
@@ -511,7 +493,25 @@
     <t>Closed by CR-003, approved 17/10/2026 by the team (E. Lindsay, Team Lead) at M4 closure; not validated with a client stakeholder. FR-6.7's measurement basis (Functional Requirements v0.3) now states the one sanctioned exception: removing personal fields at the end of the retention period under PROC-001 is not an alteration of lifecycle content (status values, change types, roles, timestamps and sequence are preserved), and it is executed only by a temporary, audited database credential outside the system's interfaces. FR-6.7's text and AC-FR-6.7 are unchanged, so FR-6.7 and NFR-4.2 no longer conflict as written. PROC-001 is still run by hand only (scripts/retention/proc-001-anonymise.js; SCP-020 deferred). Evidence: docs/change/CR-003_FR-6.7_Retention_Exception_v0.2.md; PED v4.0.</t>
   </si>
   <si>
-    <t>Gaps, derived requirements and unvalidated figures carried by this baseline. Recorded rather than resolved by invention — Master Brief s.23 values honest limitations above unsupported claims of completeness | Version 0.8 (17/10/2026, M4 final pass, R. van der Merwe). Adds columns I (Final status, M4: Closed with evidence, or Remains open for future work) and J (the engineering reason and the evidence). Every open item is given a final status. OI-05, OI-06, OI-09, OI-11 and OI-19 were closed earlier and are left exactly as they were. Adds two rows for items carried from M2 that are not open items but need a final status here: C-05 (PED Appendix B) and CON-019. E. Lindsay's two proposed items (the missing category list; the Information Officer in AC-NFR-4.5) were not raised in this version. On 18/10/2026 OI-13 was closed with evidence (CR-003 approved, PR #137; J17 in E. Lindsay's wording) and CON-019's final status confirmed from the v4.0-M4-rc evidence. Columns B to H of every existing row are unchanged. Version 0.7 (13/10/2026). Closes OI-19 (DEC-003 v0.3, PR #92, records the test environment's name, Atlas project and redacted cluster hostname separately, and the integration-test guard cites it), raised by E. Lindsay. Adds OI-21 (DEC-003 places staging and production on a VPS that never existed; found at deployment and resolved for staging only by a disposable Azure VM, with DEC-003 to be superseded), raised by R. van der Merwe. OI-01 to OI-18 and OI-20 unchanged. Version 0.6 (12/10/2026; OI-20 added 13/10/2026). Adds OI-17 (the read endpoint refuses the whole read of a security-category request to non-Security-Officer staff, which is wider than FR-1.5's three restricted fields), OI-18 (whether a blank or whitespace-only reason counts as a recorded reason under FR-6.6), OI-19 (DEC-003 names the test environment's Atlas project civicconnect-test, but the test cluster's host and the integration-test guard use civicconnecttest) and OI-20 (no CI gate inspects content inside non-Office binaries such as images and PDFs; found when an embedded provenance manifest in the three PED architecture figures passed every required check, removed on PR #94), all raised by E. Lindsay; OI-01 to OI-16 unchanged. Version 0.5 (30/09/2026). Adds OI-16 (FR-1.5 against FR-3.5/FR-3.6: whether a requester may see their own description on a security-category request), raised by E. Lindsay; OI-01 to OI-15 unchanged. Version 0.4 (30/09/2026). Adds OI-14 (reportingCounts reconciliation, owner R. van der Merwe for M3) and OI-15 (transition model confirmation, including whether a reopened-then-resolved request satisfies FR-6.5), both raised in PR #62 (E. Lindsay) and its review (R. van der Merwe). OI-01 to OI-13 are unchanged from v0.3. Version 0.3 (29/09/2026). Consolidates the M2 updates drafted by E. Lindsay (OI-05 closed; OI-06 escalated; OI-07, OI-10 updated; OI-12 raised), first committed inside the file named Open_Items_v0.2 (archived in Outdated/ and carrying those v0.3 labels), with the DEC-017 and storage updates by R. van der Merwe (OI-06 closed, OI-10 reduced, OI-13 raised). No separately committed v0.2 content exists in the repository.</t>
+    <t>FR-8.4 is now built and Met at the frozen build 6408ab7: the Manager sets a category's target resolution time, it is shown on the Categories page (DEF-028 fixed), and overdue requests are identified against it (FR-8.3 Met). What this item asks is still not done: Member A never confirmed FR-8.4 as part of SCP-011 or recorded it as new scope, so FR-8.4 stays Proposed. Evidence: RTM v0.11 (FR-8.3, FR-8.4); Scope Baseline v0.3.</t>
+  </si>
+  <si>
+    <t>FR-9.1 is now built and Met at 6408ab7: the Administrator deactivates a category from the user interface, and it is no longer offered on the New request form (E2E-7; DEF-025 fixed). Reactivation is not built. What this item asks is still not done: FR-9.1 was never confirmed as within SCP-002 or recorded as new scope. Evidence: RTM v0.11 (FR-9.1); Scope Baseline v0.3.</t>
+  </si>
+  <si>
+    <t>The response-time targets (3 s, 2 s, 5 s) and the 99 % availability figure were never confirmed with STK-005 or STK-010. At M3, NFR-2.4 passed on staging (15/10/2026, a workload without submissions). At the release candidate (18/10/2026), NFR-2.4 and NFR-2.1 were run on staging and are Not Met (DEF-032: counter contention under concurrent submissions). NFR-2.3 and NFR-2.5 were not measured. Evidence: docs/evidence/M4-perf/; RTM v0.11 (NFR-2.1, NFR-2.4).</t>
+  </si>
+  <si>
+    <t>The BC Desktop browser set was never confirmed. At M4 the E2E journeys ran 56 of 56 in four browser projects (Chromium, Chrome, Edge and Playwright's Firefox) at 6408ab7. AC-NFR-1.1 is Partially Met: prior releases and Mozilla's release Firefox are not shown, and without the BC image's set the coverage target itself is unconfirmed. Evidence: e2e/playwright.config.js; docs/evidence/M4-build/E2E_run_2026-10-17_final_four_browsers_run2.txt; RTM v0.11 (NFR-1.1).</t>
+  </si>
+  <si>
+    <t>No reconciliation job was built, and the M3 target was missed (owner R. van der Merwe). The reportingCounts projection is not registered (TD-001 partly repaid: the notification subscriber is), and the management view built at M4 counts from requests directly (FR-8.1 to FR-8.6 Met at 6408ab7), so there is no projection to drift or rebuild. The item stays open because DEC-011 and DEC-010 still describe the projection and its rebuild after a restore. scripts/backup/consistency-check.js exists for the restore path but is not scheduled. Evidence: RTM v0.11 (FR-8.1 to FR-8.6); TD-001 (Technical Debt Register v0.4); src/composition.js.</t>
+  </si>
+  <si>
+    <t>Not decided. At v4.0-M4-rc, a whitespace-only reason is still accepted: hasReason is Boolean(reason) (src/services/statusTransitionService.js line 83), and the route does not trim it. Consequence: a rejection can carry a reason that tells the requester nothing (FR-3.4). Evidence: that line; AC-FR-6.6.</t>
+  </si>
+  <si>
+    <t>Gaps, derived requirements and unvalidated figures carried by this baseline. Recorded rather than resolved by invention — Master Brief s.23 values honest limitations above unsupported claims of completeness | Version 0.8 (17/10/2026, M4 final pass, R. van der Merwe). Adds columns I (Final status, M4: Closed with evidence, or Remains open for future work) and J (the engineering reason and the evidence). Every open item is given a final status. OI-05, OI-06, OI-09, OI-11 and OI-19 were closed earlier and are left exactly as they were. Adds two rows for items carried from M2 that are not open items but need a final status here: C-05 (PED Appendix B) and CON-019. E. Lindsay's two proposed items (the missing category list; the Information Officer in AC-NFR-4.5) were not raised in this version. On 18/10/2026 OI-13 was closed with evidence (CR-003 approved, PR #137; J17 in E. Lindsay's wording) and CON-019's final status confirmed from the v4.0-M4-rc evidence. After review (18/10/2026), the reasons for OI-02, OI-03, OI-04, OI-07, OI-14 and OI-18 were brought up to date with the M4 build and the release-candidate results. Columns B to H of every existing row are unchanged. Version 0.7 (13/10/2026). Closes OI-19 (DEC-003 v0.3, PR #92, records the test environment's name, Atlas project and redacted cluster hostname separately, and the integration-test guard cites it), raised by E. Lindsay. Adds OI-21 (DEC-003 places staging and production on a VPS that never existed; found at deployment and resolved for staging only by a disposable Azure VM, with DEC-003 to be superseded), raised by R. van der Merwe. OI-01 to OI-18 and OI-20 unchanged. Version 0.6 (12/10/2026; OI-20 added 13/10/2026). Adds OI-17 (the read endpoint refuses the whole read of a security-category request to non-Security-Officer staff, which is wider than FR-1.5's three restricted fields), OI-18 (whether a blank or whitespace-only reason counts as a recorded reason under FR-6.6), OI-19 (DEC-003 names the test environment's Atlas project civicconnect-test, but the test cluster's host and the integration-test guard use civicconnecttest) and OI-20 (no CI gate inspects content inside non-Office binaries such as images and PDFs; found when an embedded provenance manifest in the three PED architecture figures passed every required check, removed on PR #94), all raised by E. Lindsay; OI-01 to OI-16 unchanged. Version 0.5 (30/09/2026). Adds OI-16 (FR-1.5 against FR-3.5/FR-3.6: whether a requester may see their own description on a security-category request), raised by E. Lindsay; OI-01 to OI-15 unchanged. Version 0.4 (30/09/2026). Adds OI-14 (reportingCounts reconciliation, owner R. van der Merwe for M3) and OI-15 (transition model confirmation, including whether a reopened-then-resolved request satisfies FR-6.5), both raised in PR #62 (E. Lindsay) and its review (R. van der Merwe). OI-01 to OI-13 are unchanged from v0.3. Version 0.3 (29/09/2026). Consolidates the M2 updates drafted by E. Lindsay (OI-05 closed; OI-06 escalated; OI-07, OI-10 updated; OI-12 raised), first committed inside the file named Open_Items_v0.2 (archived in Outdated/ and carrying those v0.3 labels), with the DEC-017 and storage updates by R. van der Merwe (OI-06 closed, OI-10 reduced, OI-13 raised). No separately committed v0.2 content exists in the repository.</t>
   </si>
 </sst>
 </file>
@@ -1061,7 +1061,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="6" spans="2:10" ht="57" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
         <v>15</v>
       </c>
@@ -1087,10 +1087,10 @@
         <v>130</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" ht="57" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
         <v>20</v>
       </c>
@@ -1116,10 +1116,10 @@
         <v>130</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="8" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" ht="99.75" x14ac:dyDescent="0.25">
       <c r="B8" s="10" t="s">
         <v>24</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>130</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>134</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
@@ -1194,7 +1194,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" ht="99.75" x14ac:dyDescent="0.25">
       <c r="B11" s="10" t="s">
         <v>44</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>130</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>135</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="2:10" ht="85.5" x14ac:dyDescent="0.25">
@@ -1249,7 +1249,7 @@
         <v>130</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" spans="2:10" ht="57" x14ac:dyDescent="0.25">
@@ -1301,7 +1301,7 @@
         <v>130</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="2:10" ht="57" x14ac:dyDescent="0.25">
@@ -1353,7 +1353,7 @@
         <v>130</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="2:10" ht="195" x14ac:dyDescent="0.25">
@@ -1379,13 +1379,13 @@
         <v>14</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="18" spans="2:10" ht="105" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" ht="150" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
         <v>83</v>
       </c>
@@ -1411,7 +1411,7 @@
         <v>130</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>139</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="225" x14ac:dyDescent="0.25">
@@ -1440,7 +1440,7 @@
         <v>130</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="20" spans="2:10" ht="90" x14ac:dyDescent="0.25">
@@ -1469,7 +1469,7 @@
         <v>130</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="2:10" ht="150" x14ac:dyDescent="0.25">
@@ -1498,7 +1498,7 @@
         <v>130</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
     </row>
     <row r="22" spans="2:10" ht="120" x14ac:dyDescent="0.25">
@@ -1527,7 +1527,7 @@
         <v>130</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>143</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="2:10" ht="345" x14ac:dyDescent="0.25">
@@ -1579,7 +1579,7 @@
         <v>130</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" spans="2:10" ht="330" x14ac:dyDescent="0.25">
@@ -1605,30 +1605,30 @@
         <v>14</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="26" spans="2:10" ht="120" x14ac:dyDescent="0.25">
       <c r="B26" s="4" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="H26" s="8" t="s">
         <v>14</v>
@@ -1637,27 +1637,27 @@
         <v>130</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="2:10" ht="165" x14ac:dyDescent="0.25">
       <c r="B27" s="4" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="H27" s="8" t="s">
         <v>14</v>
@@ -1666,7 +1666,7 @@
         <v>130</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">

</xml_diff>